<commit_message>
updated res stored in xlsx
</commit_message>
<xml_diff>
--- a/notebook/dataset/Triage-Module-Evaluation-Results.xlsx
+++ b/notebook/dataset/Triage-Module-Evaluation-Results.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,36 +425,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F150"/>
+  <dimension ref="A1:F168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>prompts</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>language</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>llm_normalized_output</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>llm_detected_language</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Detected Language</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Normalized Output</t>
         </is>
@@ -492,7 +504,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>I was not permitted to take a 3-month leave by my employer.</t>
+          <t>The employee was not permitted to take a 3-month leave of absence.</t>
         </is>
       </c>
     </row>
@@ -564,7 +576,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>I was presented with a contract different from what was discussed with the agency.</t>
+          <t>I was signed to a contract different from the one discussed with the agency.</t>
         </is>
       </c>
     </row>
@@ -588,7 +600,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>What is the legal basis for deducting my salary for meals?</t>
+          <t>What is the legal basis for deducting my salary for food?</t>
         </is>
       </c>
     </row>
@@ -660,7 +672,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Can an employer detain an employee if they flee?</t>
+          <t>Can an employer imprison an employee if they flee?</t>
         </is>
       </c>
     </row>
@@ -708,7 +720,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>The contract has been completed but the party is refusing to allow the employee to return.</t>
+          <t>The contract has been completed but the party is refusing to allow the return.</t>
         </is>
       </c>
     </row>
@@ -900,7 +912,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>I am being forced to sleep on the kitchen floor, can this be reported?</t>
+          <t>I am sleeping on the kitchen floor, can that be reported?</t>
         </is>
       </c>
     </row>
@@ -924,7 +936,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Delayed salary for two months, what are my rights?</t>
+          <t>Delayed two months of my salary, what are my rights?</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1248,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>I am afraid to report because I might be deported.</t>
+          <t>Afraid to report, might be deported.</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1296,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>What is required for an OEC when returning briefly?</t>
+          <t>What is required for a OEC when returning briefly?</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1392,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Moved to night shift without prior notice.</t>
+          <t>I was transferred to the night shift without prior notice.</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1488,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Sent money to the agency but it was a scam.</t>
+          <t>Sent money to the agency but it turned out to be a scam.</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1536,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Can a breach of contract lawsuit be filed in the Philippines?</t>
+          <t>Can a person be sued for breach of contract in the Philippines?</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1560,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Should the embassy have the right to send me back?</t>
+          <t>Can the embassy send me back?</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1584,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>I did not receive the last payment before leaving.</t>
+          <t>I did not receive my final paycheck before leaving.</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1680,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Termination is valid if communicated through text message only?</t>
+          <t>Does the termination remain valid if it was communicated through text message only?</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1704,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>I overstayed by 2 days, will this cause problems with Immigration?</t>
+          <t>I overstayed for 2 days, will this cause problems with Immigration?</t>
         </is>
       </c>
     </row>
@@ -1716,7 +1728,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Employee's employer refuses to provide separation pay, what to do?</t>
+          <t>What to do regarding the employer's refusal to provide separation pay?</t>
         </is>
       </c>
     </row>
@@ -1740,7 +1752,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Check if the agency being spoken to is legitimate.</t>
+          <t>Check whether the agency contacted is legitimate.</t>
         </is>
       </c>
     </row>
@@ -1764,7 +1776,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Must an OFW pay tax in the Philippines?</t>
+          <t>Do OFWs need to pay taxes in the Philippines?</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1800,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Help, I am being verbally harassed by my employer, can I file a complaint?</t>
+          <t>Help me, I am being verbally harassed by my employer, can I file a complaint?</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1824,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Please advise, the party wishes to terminate the contract because of toxic conditions.</t>
+          <t>Please advise, the party wishes to terminate the contract because it is toxic.</t>
         </is>
       </c>
     </row>
@@ -1860,7 +1872,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>The employer confiscated the employee's phone. Is this permissible?</t>
+          <t>I am alleged to have had my phone confiscated by my employer.</t>
         </is>
       </c>
     </row>
@@ -1908,7 +1920,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>How to claim Long Service Payment after 5 years?</t>
+          <t>How to claim long service payment after 5 years?</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1944,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>I lost my passport, how can I return home?</t>
+          <t>I lost my passport, how can I return?</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1992,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>The agency I am associated with is requesting an additional fee, is this a scam?</t>
+          <t>The agency is requesting an additional fee, is this a scam?</t>
         </is>
       </c>
     </row>
@@ -2143,7 +2155,7 @@
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Tagalog</t>
+          <t>Taglish</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -2220,7 +2232,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>I was accused of theft without evidence, can I file a lawsuit?</t>
+          <t>I am accused of theft without evidence, can I file a lawsuit?</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2256,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>I wish to resign but has a bond.</t>
+          <t>I wish to resign but there is a bond agreement.</t>
         </is>
       </c>
     </row>
@@ -2268,7 +2280,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>I am being forced to sign a document that I do not understand.</t>
+          <t>I am being forced to sign a document I do not understand.</t>
         </is>
       </c>
     </row>
@@ -2340,7 +2352,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>I am physically abused by my employer, where should I report?</t>
+          <t>I am physically abused by my employer, where should I report it?</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2448,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>What should be done, I do not want to be given a release letter?</t>
+          <t>What should I do, I do not want to be given a release letter?</t>
         </is>
       </c>
     </row>
@@ -2484,7 +2496,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>The alleged delayed salary constitutes grounds for termination.</t>
+          <t>The employee's salary is frequently delayed, can this be grounds for termination?</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2688,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>I am awaiting departure orders, how will I know?</t>
+          <t>I was issued a hold departure order, how can I find out?</t>
         </is>
       </c>
     </row>
@@ -2700,7 +2712,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Can the spouse file an adultery case against me even if I am abroad?</t>
+          <t>Can the spouse file an adultery case if the person is abroad?</t>
         </is>
       </c>
     </row>
@@ -2820,7 +2832,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Renewal of passport pages is required at the consulate?</t>
+          <t>Renew passport pages at consulate?</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2856,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>I did not receive MPF payments from my employer. Can a report be filed?</t>
+          <t>I did not receive MPF payments, can I report?</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2880,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>The employer's failure to provide notice period prior to termination is unlawful.</t>
+          <t>The employer's failure to provide notice period before termination is illegal.</t>
         </is>
       </c>
     </row>
@@ -2892,7 +2904,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>I have worked for five years, should I be entitled to long service leave?</t>
+          <t>I have worked for five years, should I be entitled to long service money?</t>
         </is>
       </c>
     </row>
@@ -3012,7 +3024,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>If an employee works a part-time job during their vacation period, would that be illegal?</t>
+          <t>If an employee works a side job during their vacation period, would that be illegal?</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3048,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>The employer has taken the passport and refuses to return it.</t>
+          <t>I am alleged to have had my passport taken by my employer and not returned.</t>
         </is>
       </c>
     </row>
@@ -3108,7 +3120,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>I have not completed the contract, may I switch to a new employer?</t>
+          <t>I have not completed the contract, can I switch to a new employer?</t>
         </is>
       </c>
     </row>
@@ -3132,7 +3144,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>The employer did not provide insurance, what should be done when I became ill?</t>
+          <t>The employer did not provide insurance, what happens if I get sick?</t>
         </is>
       </c>
     </row>
@@ -3252,7 +3264,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>They do not provide me with enough food to eat, does this constitute abuse?</t>
+          <t>The subjects did not provide me with sufficient food, does this constitute abuse?</t>
         </is>
       </c>
     </row>
@@ -3348,7 +3360,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>What are the legal implications of debt on visa application?</t>
+          <t>What is the impact of debt on visa application?</t>
         </is>
       </c>
     </row>
@@ -3372,7 +3384,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Does the contract remain valid after the employer's death?</t>
+          <t>Does the employment contract remain valid after the employer's death?</t>
         </is>
       </c>
     </row>
@@ -3420,7 +3432,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>I was not given notice of the termination, can I pursue legal action?</t>
+          <t>I was not given notice of the severance payment, and I am seeking legal recourse.</t>
         </is>
       </c>
     </row>
@@ -3468,7 +3480,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>They installed CCTV in the restroom, I am very scared.</t>
+          <t>The alleged installation of CCTV in the restroom caused fear.</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3504,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>I am required to work 20 hours per day, which is not feasible, can I report to the labor department?</t>
+          <t>I am required to work 20 hours per day, which is unreasonable, can I report to the labor department?</t>
         </is>
       </c>
     </row>
@@ -3516,7 +3528,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>I have not received the last installment of food.</t>
+          <t>I did not receive the last installment of food.</t>
         </is>
       </c>
     </row>
@@ -3583,12 +3595,12 @@
       <c r="D132" t="inlineStr"/>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Cantonese</t>
+          <t>Chinese</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Departure is required when the visa is denied.</t>
+          <t>Departure date after visa rejection.</t>
         </is>
       </c>
     </row>
@@ -3660,7 +3672,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>The subjects do not communicate with their family members via telephone.</t>
+          <t>The individuals do not contact their family members by telephone as I do.</t>
         </is>
       </c>
     </row>
@@ -3756,7 +3768,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Go to the embassy first due to labor disputes.</t>
+          <t>What is the procedure for labor disputes? Should one go to the consulate first?</t>
         </is>
       </c>
     </row>
@@ -3804,7 +3816,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Is the injury considered a work-related injury?</t>
+          <t>If injured, is it a work-related injury?</t>
         </is>
       </c>
     </row>
@@ -3852,7 +3864,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Can a relative stay overnight?</t>
+          <t>Can the petitioner have relatives stay for one night?</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3912,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Who will pay for the ticket if the contract is terminated early?</t>
+          <t>Who pays for the ticket if the contract is terminated early?</t>
         </is>
       </c>
     </row>
@@ -3924,7 +3936,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Am I required to follow my boss to immigrate?</t>
+          <t>I am required to follow my employer to the immigration?</t>
         </is>
       </c>
     </row>
@@ -3948,7 +3960,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>No contract signed before commencement of work, is there any protection?</t>
+          <t>No contract, start work, any protection?</t>
         </is>
       </c>
     </row>
@@ -4021,6 +4033,438 @@
       <c r="F150" t="inlineStr">
         <is>
           <t>Where can free legal consultation be found?</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>我啱啱發現有咗BB，老細知道之後即刻話要炒我，香港法例係咪容許咁樣？</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr"/>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>I have just discovered that I am pregnant. My employer immediately stated that they would fire me. Does Hong Kong law allow such actions?</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>其實我做得好唔開心想自己斷約，但係我無錢賠一個月糧，可唔可以即刻走？</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr"/>
+      <c r="D152" t="inlineStr"/>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>I was not willing to terminate the contract, but I cannot afford to pay one month's salary. Can I leave immediately?</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>呢幾個月老細都係遲出糧，有時拖成十幾日，我投訴佢就話無錢，我可唔可以當佢自動解僱我？</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr"/>
+      <c r="D153" t="inlineStr"/>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>These months, the boss has been delaying payroll, sometimes up to 15 days. I complained, and he said he has no money. Can I consider him to have automatically terminated my employment?</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>每個月出糧佢都淨係俾三千幾蚊我，話扣起咗啲做中介費，但我未簽過任何同意書。</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr"/>
+      <c r="D154" t="inlineStr"/>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Every month he only gives me three thousand or so, stating that some amount has been withheld as a brokerage fee, but I have not signed any consent form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>合約寫明包食宿，但每個月都冇比膳食津貼，又要我用自己人工買餸自己煮，算唔算犯法？</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr"/>
+      <c r="D155" t="inlineStr"/>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>The contract states that accommodation and meals are provided, but no meal allowance is given each month, and the employee is required to use their own salary to buy groceries and cook, does this constitute a legal violation?</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>佢哋安排我同個十歲嘅男仔同埋老爺一間房訓，我覺得好唔舒服，勞工處有冇規定住宿環境？</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr"/>
+      <c r="D156" t="inlineStr"/>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>I was arranged to share a room with a 10-year-old boy and an elderly person, which I found uncomfortable. Does the Labour Department have regulations regarding accommodation conditions?</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>我發高燒入咗醫院，僱主話醫藥費太貴唔肯幫我比，仲話要扣我人工當醫藥費。</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr"/>
+      <c r="D157" t="inlineStr"/>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>I was hospitalized due to a high fever, and the employer stated that the medical expenses were too expensive and refused to cover them, and also stated that they would deduct my salary as medical expenses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>每日由朝早六點做到半夜一點，完全無私人時間休息，我有冇權利要求固定休息時間？</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr"/>
+      <c r="D158" t="inlineStr"/>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>I have no right to request fixed rest time if I work from 6:00 AM to 1:00 AM every day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>僱主逼我簽一份『自願離職』信，話唔簽就報警屈我偷嘢，我好驚，點算好？</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr"/>
+      <c r="D159" t="inlineStr"/>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>I am afraid and do not know what to do, as the employer is forcing me to sign a 'voluntary resignation' letter and threatened to report me for theft if I do not sign.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>做咗三個月，僱主話我做嘢太慢終止合約，佢係咪需要負責我返去嘅機票？</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr"/>
+      <c r="D160" t="inlineStr"/>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>I was employed for three months, and the employer stated that I was working too slowly and terminated the contract. Is the employer required to cover my return flight ticket?</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>僱主突然話聽日唔洗我返工，又唔補一個月代通知金比我，我依家可以點做？</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr"/>
+      <c r="D161" t="inlineStr"/>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>What can I do now that the employer suddenly said I don't have to come to work tomorrow and did not provide one month's notice pay?</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>我不小心整爛咗個微波爐，老細今個月扣咗我二千蚊人工，佢係咪可以扣咁多？</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr"/>
+      <c r="D162" t="inlineStr"/>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>I accidentally damaged a microwave, and the boss deducted 2000 Hong Kong dollars from my salary this month. Is the boss legally allowed to deduct that amount?</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>佢話我上星期表現唔好，所以今個月要扣減五百蚊人工當懲罰，勞工法例有冇話唔得？</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr"/>
+      <c r="D163" t="inlineStr"/>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>The employee claims that their work performance was poor last week, so their salary will be reduced by 500 HKD as punishment. Is there a provision in the Labour Law that prohibits this?</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>我抹緊窗嗰陣跌親隻手，但僱主冇幫我買勞保，依家唔肯負責我嘅物理治療費用，點算？</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr"/>
+      <c r="D164" t="inlineStr"/>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>I suffered a hand injury while cleaning the window, but the employer did not purchase labor insurance, and now refuses to cover the physical therapy expenses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>老細成日用粗口鬧我，有時仲會掟嘢，我覺得人身安全受威脅，佢咁做算唔算違反僱傭合約？</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr"/>
+      <c r="D165" t="inlineStr"/>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>I allege that the employer used vulgar language and threw objects, and I believe my personal safety is threatened. Does this constitute a breach of the employment contract?</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>老細叫我星期日放假都要留喺屋企照顧小朋友，話補返一百蚊比我，我可唔可以拒絕？</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr"/>
+      <c r="D166" t="inlineStr"/>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>I can refuse the employer's request to stay at home on Sunday to take care of the children, as the employer offered to compensate me with 100 HKD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>婆婆（受照顧者）過身，佢個仔話合約即刻完，要我聽日就買機票返菲律賓，咁我啲遣散費點計？</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr"/>
+      <c r="D167" t="inlineStr"/>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>The deceased (care recipient) passed away, and her son stated that the contract is immediately terminated, requiring me to purchase a ticket back to the Philippines tomorrow. How is my severance pay calculated?</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>我平時除咗做家務，老細仲日日叫我落去佢間茶餐廳幫手洗碗，咁樣係咪做緊黑工？</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr"/>
+      <c r="D168" t="inlineStr"/>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>I routinely assist with household chores and the employer regularly asks me to work at his restaurant washing dishes. Is this considered illegal labor?</t>
         </is>
       </c>
     </row>

</xml_diff>